<commit_message>
Split agent run 9 for min model 14. simplified reward on actions. fixed a bug on the test win rate for the next runs.
</commit_message>
<xml_diff>
--- a/startegies/COMPARE_TO_IDEAL.xlsx
+++ b/startegies/COMPARE_TO_IDEAL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Python\BLACKJACK-AI\BlackJack-1.1.26\startegies\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Python\BLACKJACK-AI\BlackJack\startegies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07EAB49A-8D97-4E18-8131-495D7628D531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F680A3CC-1077-4234-BA3A-A2BB4644DE41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14385" yWindow="240" windowWidth="14250" windowHeight="15105" firstSheet="7" activeTab="10" xr2:uid="{7D4E3D51-C410-42E7-8E6F-E5B372043018}"/>
+    <workbookView xWindow="-14385" yWindow="240" windowWidth="14250" windowHeight="15105" firstSheet="7" activeTab="11" xr2:uid="{7D4E3D51-C410-42E7-8E6F-E5B372043018}"/>
   </bookViews>
   <sheets>
     <sheet name="IDEAL_STRAT" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="strat_14_6" sheetId="9" r:id="rId9"/>
     <sheet name="strat_14_7" sheetId="10" r:id="rId10"/>
     <sheet name="strat_14_8" sheetId="11" r:id="rId11"/>
+    <sheet name="strat_14_9" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="6">
   <si>
     <t>HARD HANDS - NO PAIRS</t>
   </si>
@@ -129,28 +130,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="15">
     <dxf>
       <fill>
         <patternFill>
@@ -1940,39 +1920,24 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A49:K51">
-    <cfRule type="expression" dxfId="15" priority="7">
-      <formula>A49:K93&lt;&gt;A49:K93</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1">
-    <cfRule type="expression" dxfId="14" priority="6">
+  <conditionalFormatting sqref="A1:A2">
+    <cfRule type="expression" dxfId="14" priority="5">
       <formula>A1:K45&lt;&gt;A1:K45</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2">
-    <cfRule type="expression" dxfId="13" priority="5">
-      <formula>A2:K46&lt;&gt;A2:K46</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A21">
-    <cfRule type="expression" dxfId="12" priority="4">
+  <conditionalFormatting sqref="A21:A22">
+    <cfRule type="expression" dxfId="13" priority="3">
       <formula>A21:K65&lt;&gt;A21:K65</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A22">
-    <cfRule type="expression" dxfId="11" priority="3">
-      <formula>A22:K66&lt;&gt;A22:K66</formula>
+  <conditionalFormatting sqref="A34:A35">
+    <cfRule type="expression" dxfId="12" priority="1">
+      <formula>A34:K78&lt;&gt;A34:K78</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A35">
-    <cfRule type="expression" dxfId="10" priority="2">
-      <formula>A35:K79&lt;&gt;A35:K79</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A34">
-    <cfRule type="expression" dxfId="9" priority="1">
-      <formula>A34:K78&lt;&gt;A34:K78</formula>
+  <conditionalFormatting sqref="A49:K51">
+    <cfRule type="expression" dxfId="11" priority="7">
+      <formula>A49:K93&lt;&gt;A49:K93</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4740,6 +4705,1386 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC61F169-432C-4CAE-B0DF-B80B8CF95B47}">
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>6</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>9</v>
+      </c>
+      <c r="J2">
+        <v>10</v>
+      </c>
+      <c r="K2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>4</v>
+      </c>
+      <c r="J13">
+        <v>4</v>
+      </c>
+      <c r="K13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14">
+        <v>3</v>
+      </c>
+      <c r="H14">
+        <v>4</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+      <c r="J14">
+        <v>4</v>
+      </c>
+      <c r="K14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>3</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>3</v>
+      </c>
+      <c r="K15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
+      <c r="K16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="F22">
+        <v>6</v>
+      </c>
+      <c r="G22">
+        <v>7</v>
+      </c>
+      <c r="H22">
+        <v>8</v>
+      </c>
+      <c r="I22">
+        <v>9</v>
+      </c>
+      <c r="J22">
+        <v>10</v>
+      </c>
+      <c r="K22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>13</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>14</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>15</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>16</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>17</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>18</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>3</v>
+      </c>
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+      <c r="I28">
+        <v>3</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>19</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29">
+        <v>3</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+      <c r="F29">
+        <v>3</v>
+      </c>
+      <c r="G29">
+        <v>3</v>
+      </c>
+      <c r="H29">
+        <v>3</v>
+      </c>
+      <c r="I29">
+        <v>3</v>
+      </c>
+      <c r="J29">
+        <v>3</v>
+      </c>
+      <c r="K29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>20</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <v>3</v>
+      </c>
+      <c r="H30">
+        <v>3</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="K30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35">
+        <v>6</v>
+      </c>
+      <c r="G35">
+        <v>7</v>
+      </c>
+      <c r="H35">
+        <v>8</v>
+      </c>
+      <c r="I35">
+        <v>9</v>
+      </c>
+      <c r="J35">
+        <v>10</v>
+      </c>
+      <c r="K35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>2</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="E36">
+        <v>2</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36">
+        <v>2</v>
+      </c>
+      <c r="H36">
+        <v>2</v>
+      </c>
+      <c r="I36">
+        <v>2</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>3</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37">
+        <v>2</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38">
+        <v>1</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>5</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39">
+        <v>0</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>6</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40">
+        <v>2</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
+      <c r="G40">
+        <v>2</v>
+      </c>
+      <c r="H40">
+        <v>2</v>
+      </c>
+      <c r="I40">
+        <v>2</v>
+      </c>
+      <c r="J40">
+        <v>2</v>
+      </c>
+      <c r="K40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>7</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41">
+        <v>2</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+      <c r="G41">
+        <v>2</v>
+      </c>
+      <c r="H41">
+        <v>2</v>
+      </c>
+      <c r="I41">
+        <v>2</v>
+      </c>
+      <c r="J41">
+        <v>2</v>
+      </c>
+      <c r="K41">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>8</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42">
+        <v>2</v>
+      </c>
+      <c r="H42">
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>2</v>
+      </c>
+      <c r="J42">
+        <v>2</v>
+      </c>
+      <c r="K42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>9</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43">
+        <v>2</v>
+      </c>
+      <c r="F43">
+        <v>2</v>
+      </c>
+      <c r="G43">
+        <v>3</v>
+      </c>
+      <c r="H43">
+        <v>2</v>
+      </c>
+      <c r="I43">
+        <v>2</v>
+      </c>
+      <c r="J43">
+        <v>2</v>
+      </c>
+      <c r="K43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>10</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44">
+        <v>3</v>
+      </c>
+      <c r="E44">
+        <v>3</v>
+      </c>
+      <c r="F44">
+        <v>3</v>
+      </c>
+      <c r="G44">
+        <v>3</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44">
+        <v>3</v>
+      </c>
+      <c r="K44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>11</v>
+      </c>
+      <c r="B45">
+        <v>2</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>2</v>
+      </c>
+      <c r="G45">
+        <v>2</v>
+      </c>
+      <c r="H45">
+        <v>2</v>
+      </c>
+      <c r="I45">
+        <v>2</v>
+      </c>
+      <c r="J45">
+        <v>2</v>
+      </c>
+      <c r="K45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="D50">
+        <v>4</v>
+      </c>
+      <c r="E50">
+        <v>5</v>
+      </c>
+      <c r="F50">
+        <v>6</v>
+      </c>
+      <c r="G50">
+        <v>7</v>
+      </c>
+      <c r="H50">
+        <v>8</v>
+      </c>
+      <c r="I50">
+        <v>9</v>
+      </c>
+      <c r="J50">
+        <v>10</v>
+      </c>
+      <c r="K50">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
+      </c>
+      <c r="D51">
+        <v>3</v>
+      </c>
+      <c r="E51">
+        <v>3</v>
+      </c>
+      <c r="F51">
+        <v>3</v>
+      </c>
+      <c r="G51">
+        <v>3</v>
+      </c>
+      <c r="H51">
+        <v>3</v>
+      </c>
+      <c r="I51">
+        <v>3</v>
+      </c>
+      <c r="J51">
+        <v>3</v>
+      </c>
+      <c r="K51">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="1" id="{518CA509-3642-4190-8AA4-712C99EF57A3}">
+            <xm:f>A1:K45&lt;&gt;IDEAL_STRAT!A1:K45</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>A1:K51</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{937B308A-3064-4D2F-B194-556AEB25218E}">
   <dimension ref="A1:K51"/>

</xml_diff>

<commit_message>
Split model no.10 - simplified action rewards some more
</commit_message>
<xml_diff>
--- a/startegies/COMPARE_TO_IDEAL.xlsx
+++ b/startegies/COMPARE_TO_IDEAL.xlsx
@@ -8,9 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Python\BLACKJACK-AI\BlackJack\startegies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F680A3CC-1077-4234-BA3A-A2BB4644DE41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC8F248-F440-464C-9496-6ECB691D8B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14385" yWindow="240" windowWidth="14250" windowHeight="15105" firstSheet="7" activeTab="11" xr2:uid="{7D4E3D51-C410-42E7-8E6F-E5B372043018}"/>
+    <workbookView xWindow="-14385" yWindow="240" windowWidth="14250" windowHeight="15105" firstSheet="9" activeTab="12" xr2:uid="{7D4E3D51-C410-42E7-8E6F-E5B372043018}"/>
+    <workbookView minimized="1" xWindow="-28725" yWindow="285" windowWidth="14250" windowHeight="15105" xr2:uid="{B4A4BA22-06B5-4DC4-A625-CB67E331C3A1}"/>
   </bookViews>
   <sheets>
     <sheet name="IDEAL_STRAT" sheetId="1" r:id="rId1"/>
@@ -25,6 +26,7 @@
     <sheet name="strat_14_7" sheetId="10" r:id="rId10"/>
     <sheet name="strat_14_8" sheetId="11" r:id="rId11"/>
     <sheet name="strat_14_9" sheetId="12" r:id="rId12"/>
+    <sheet name="strat_14_10" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="6">
   <si>
     <t>HARD HANDS - NO PAIRS</t>
   </si>
@@ -130,7 +132,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1569,13 +1578,13 @@
         <v>4</v>
       </c>
       <c r="B38" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C38" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D38" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E38" s="1">
         <v>2</v>
@@ -1921,22 +1930,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A2">
-    <cfRule type="expression" dxfId="14" priority="5">
+    <cfRule type="expression" dxfId="15" priority="5">
       <formula>A1:K45&lt;&gt;A1:K45</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A21:A22">
-    <cfRule type="expression" dxfId="13" priority="3">
+    <cfRule type="expression" dxfId="14" priority="3">
       <formula>A21:K65&lt;&gt;A21:K65</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A34:A35">
-    <cfRule type="expression" dxfId="12" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>A34:K78&lt;&gt;A34:K78</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A49:K51">
-    <cfRule type="expression" dxfId="11" priority="7">
+    <cfRule type="expression" dxfId="12" priority="7">
       <formula>A49:K93&lt;&gt;A49:K93</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6085,6 +6094,1386 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{871AA6C2-75D9-4897-84A3-B6598DF5AE56}">
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>6</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>9</v>
+      </c>
+      <c r="J2">
+        <v>10</v>
+      </c>
+      <c r="K2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>4</v>
+      </c>
+      <c r="J13">
+        <v>4</v>
+      </c>
+      <c r="K13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14">
+        <v>3</v>
+      </c>
+      <c r="H14">
+        <v>4</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+      <c r="J14">
+        <v>4</v>
+      </c>
+      <c r="K14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>3</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>3</v>
+      </c>
+      <c r="K15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
+      <c r="K16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="F22">
+        <v>6</v>
+      </c>
+      <c r="G22">
+        <v>7</v>
+      </c>
+      <c r="H22">
+        <v>8</v>
+      </c>
+      <c r="I22">
+        <v>9</v>
+      </c>
+      <c r="J22">
+        <v>10</v>
+      </c>
+      <c r="K22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>13</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>14</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>15</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>16</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>17</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>18</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>3</v>
+      </c>
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+      <c r="I28">
+        <v>3</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>19</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29">
+        <v>3</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+      <c r="F29">
+        <v>3</v>
+      </c>
+      <c r="G29">
+        <v>3</v>
+      </c>
+      <c r="H29">
+        <v>3</v>
+      </c>
+      <c r="I29">
+        <v>3</v>
+      </c>
+      <c r="J29">
+        <v>3</v>
+      </c>
+      <c r="K29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>20</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <v>3</v>
+      </c>
+      <c r="H30">
+        <v>3</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="K30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35">
+        <v>6</v>
+      </c>
+      <c r="G35">
+        <v>7</v>
+      </c>
+      <c r="H35">
+        <v>8</v>
+      </c>
+      <c r="I35">
+        <v>9</v>
+      </c>
+      <c r="J35">
+        <v>10</v>
+      </c>
+      <c r="K35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>2</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="E36">
+        <v>2</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36">
+        <v>2</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>2</v>
+      </c>
+      <c r="K36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>3</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37">
+        <v>2</v>
+      </c>
+      <c r="H37">
+        <v>2</v>
+      </c>
+      <c r="I37">
+        <v>2</v>
+      </c>
+      <c r="J37">
+        <v>2</v>
+      </c>
+      <c r="K37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>2</v>
+      </c>
+      <c r="D38">
+        <v>2</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>2</v>
+      </c>
+      <c r="H38">
+        <v>2</v>
+      </c>
+      <c r="I38">
+        <v>2</v>
+      </c>
+      <c r="J38">
+        <v>2</v>
+      </c>
+      <c r="K38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>5</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39">
+        <v>0</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>6</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40">
+        <v>2</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
+      <c r="G40">
+        <v>2</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>7</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41">
+        <v>2</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+      <c r="G41">
+        <v>2</v>
+      </c>
+      <c r="H41">
+        <v>2</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>8</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42">
+        <v>2</v>
+      </c>
+      <c r="H42">
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>2</v>
+      </c>
+      <c r="J42">
+        <v>2</v>
+      </c>
+      <c r="K42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>9</v>
+      </c>
+      <c r="B43">
+        <v>2</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43">
+        <v>3</v>
+      </c>
+      <c r="F43">
+        <v>3</v>
+      </c>
+      <c r="G43">
+        <v>3</v>
+      </c>
+      <c r="H43">
+        <v>3</v>
+      </c>
+      <c r="I43">
+        <v>2</v>
+      </c>
+      <c r="J43">
+        <v>3</v>
+      </c>
+      <c r="K43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>10</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44">
+        <v>3</v>
+      </c>
+      <c r="E44">
+        <v>3</v>
+      </c>
+      <c r="F44">
+        <v>3</v>
+      </c>
+      <c r="G44">
+        <v>3</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44">
+        <v>3</v>
+      </c>
+      <c r="K44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>11</v>
+      </c>
+      <c r="B45">
+        <v>2</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>2</v>
+      </c>
+      <c r="G45">
+        <v>2</v>
+      </c>
+      <c r="H45">
+        <v>2</v>
+      </c>
+      <c r="I45">
+        <v>2</v>
+      </c>
+      <c r="J45">
+        <v>2</v>
+      </c>
+      <c r="K45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="D50">
+        <v>4</v>
+      </c>
+      <c r="E50">
+        <v>5</v>
+      </c>
+      <c r="F50">
+        <v>6</v>
+      </c>
+      <c r="G50">
+        <v>7</v>
+      </c>
+      <c r="H50">
+        <v>8</v>
+      </c>
+      <c r="I50">
+        <v>9</v>
+      </c>
+      <c r="J50">
+        <v>10</v>
+      </c>
+      <c r="K50">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
+      </c>
+      <c r="D51">
+        <v>3</v>
+      </c>
+      <c r="E51">
+        <v>3</v>
+      </c>
+      <c r="F51">
+        <v>3</v>
+      </c>
+      <c r="G51">
+        <v>3</v>
+      </c>
+      <c r="H51">
+        <v>3</v>
+      </c>
+      <c r="I51">
+        <v>3</v>
+      </c>
+      <c r="J51">
+        <v>3</v>
+      </c>
+      <c r="K51">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="1" id="{E2F37819-5BB2-47D2-8EDE-0B8AFA0904DD}">
+            <xm:f>A1:K45&lt;&gt;IDEAL_STRAT!A1:K45</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>A1:K51</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{937B308A-3064-4D2F-B194-556AEB25218E}">
   <dimension ref="A1:K51"/>

</xml_diff>

<commit_message>
Split model no.11 for Min model no.14.
</commit_message>
<xml_diff>
--- a/startegies/COMPARE_TO_IDEAL.xlsx
+++ b/startegies/COMPARE_TO_IDEAL.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Python\BLACKJACK-AI\BlackJack\startegies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC8F248-F440-464C-9496-6ECB691D8B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8624736-EFBB-428D-A55C-AC4BAE7BC2D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14385" yWindow="240" windowWidth="14250" windowHeight="15105" firstSheet="9" activeTab="12" xr2:uid="{7D4E3D51-C410-42E7-8E6F-E5B372043018}"/>
-    <workbookView minimized="1" xWindow="-28725" yWindow="285" windowWidth="14250" windowHeight="15105" xr2:uid="{B4A4BA22-06B5-4DC4-A625-CB67E331C3A1}"/>
+    <workbookView xWindow="-14385" yWindow="240" windowWidth="14250" windowHeight="15105" firstSheet="12" activeTab="14" xr2:uid="{7D4E3D51-C410-42E7-8E6F-E5B372043018}"/>
+    <workbookView xWindow="-28665" yWindow="240" windowWidth="14250" windowHeight="15105" xr2:uid="{D3AF0EBA-7B40-4C08-87C2-5ACC0D5D261F}"/>
   </bookViews>
   <sheets>
     <sheet name="IDEAL_STRAT" sheetId="1" r:id="rId1"/>
@@ -27,6 +27,8 @@
     <sheet name="strat_14_8" sheetId="11" r:id="rId11"/>
     <sheet name="strat_14_9" sheetId="12" r:id="rId12"/>
     <sheet name="strat_14_10" sheetId="13" r:id="rId13"/>
+    <sheet name="strat_14_11" sheetId="14" r:id="rId14"/>
+    <sheet name="strat_14_11 (2)" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="6">
   <si>
     <t>HARD HANDS - NO PAIRS</t>
   </si>
@@ -132,7 +134,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="18">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1930,22 +1946,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A2">
-    <cfRule type="expression" dxfId="15" priority="5">
+    <cfRule type="expression" dxfId="17" priority="5">
       <formula>A1:K45&lt;&gt;A1:K45</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A21:A22">
-    <cfRule type="expression" dxfId="14" priority="3">
+    <cfRule type="expression" dxfId="16" priority="3">
       <formula>A21:K65&lt;&gt;A21:K65</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A34:A35">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="15" priority="1">
       <formula>A34:K78&lt;&gt;A34:K78</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A49:K51">
-    <cfRule type="expression" dxfId="12" priority="7">
+    <cfRule type="expression" dxfId="14" priority="7">
       <formula>A49:K93&lt;&gt;A49:K93</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7474,6 +7490,2766 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49F6F120-9B50-4F37-864F-1DABED99D7F0}">
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>6</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>9</v>
+      </c>
+      <c r="J2">
+        <v>10</v>
+      </c>
+      <c r="K2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>4</v>
+      </c>
+      <c r="J13">
+        <v>4</v>
+      </c>
+      <c r="K13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14">
+        <v>3</v>
+      </c>
+      <c r="H14">
+        <v>4</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+      <c r="J14">
+        <v>4</v>
+      </c>
+      <c r="K14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>3</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>3</v>
+      </c>
+      <c r="K15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
+      <c r="K16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="F22">
+        <v>6</v>
+      </c>
+      <c r="G22">
+        <v>7</v>
+      </c>
+      <c r="H22">
+        <v>8</v>
+      </c>
+      <c r="I22">
+        <v>9</v>
+      </c>
+      <c r="J22">
+        <v>10</v>
+      </c>
+      <c r="K22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>13</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>14</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>15</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>16</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>17</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>18</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>3</v>
+      </c>
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+      <c r="I28">
+        <v>3</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>19</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29">
+        <v>3</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+      <c r="F29">
+        <v>3</v>
+      </c>
+      <c r="G29">
+        <v>3</v>
+      </c>
+      <c r="H29">
+        <v>3</v>
+      </c>
+      <c r="I29">
+        <v>3</v>
+      </c>
+      <c r="J29">
+        <v>3</v>
+      </c>
+      <c r="K29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>20</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <v>3</v>
+      </c>
+      <c r="H30">
+        <v>3</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="K30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35">
+        <v>6</v>
+      </c>
+      <c r="G35">
+        <v>7</v>
+      </c>
+      <c r="H35">
+        <v>8</v>
+      </c>
+      <c r="I35">
+        <v>9</v>
+      </c>
+      <c r="J35">
+        <v>10</v>
+      </c>
+      <c r="K35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>2</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="E36">
+        <v>2</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>3</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>5</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39">
+        <v>0</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>6</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40">
+        <v>2</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
+      <c r="G40">
+        <v>2</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>7</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41">
+        <v>2</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+      <c r="G41">
+        <v>2</v>
+      </c>
+      <c r="H41">
+        <v>2</v>
+      </c>
+      <c r="I41">
+        <v>2</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>8</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42">
+        <v>2</v>
+      </c>
+      <c r="H42">
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>2</v>
+      </c>
+      <c r="J42">
+        <v>2</v>
+      </c>
+      <c r="K42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>9</v>
+      </c>
+      <c r="B43">
+        <v>2</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43">
+        <v>2</v>
+      </c>
+      <c r="F43">
+        <v>3</v>
+      </c>
+      <c r="G43">
+        <v>3</v>
+      </c>
+      <c r="H43">
+        <v>2</v>
+      </c>
+      <c r="I43">
+        <v>2</v>
+      </c>
+      <c r="J43">
+        <v>3</v>
+      </c>
+      <c r="K43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>10</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44">
+        <v>3</v>
+      </c>
+      <c r="E44">
+        <v>3</v>
+      </c>
+      <c r="F44">
+        <v>3</v>
+      </c>
+      <c r="G44">
+        <v>3</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44">
+        <v>3</v>
+      </c>
+      <c r="K44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>11</v>
+      </c>
+      <c r="B45">
+        <v>2</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>2</v>
+      </c>
+      <c r="G45">
+        <v>2</v>
+      </c>
+      <c r="H45">
+        <v>2</v>
+      </c>
+      <c r="I45">
+        <v>2</v>
+      </c>
+      <c r="J45">
+        <v>2</v>
+      </c>
+      <c r="K45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="D50">
+        <v>4</v>
+      </c>
+      <c r="E50">
+        <v>5</v>
+      </c>
+      <c r="F50">
+        <v>6</v>
+      </c>
+      <c r="G50">
+        <v>7</v>
+      </c>
+      <c r="H50">
+        <v>8</v>
+      </c>
+      <c r="I50">
+        <v>9</v>
+      </c>
+      <c r="J50">
+        <v>10</v>
+      </c>
+      <c r="K50">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
+      </c>
+      <c r="D51">
+        <v>3</v>
+      </c>
+      <c r="E51">
+        <v>3</v>
+      </c>
+      <c r="F51">
+        <v>3</v>
+      </c>
+      <c r="G51">
+        <v>3</v>
+      </c>
+      <c r="H51">
+        <v>3</v>
+      </c>
+      <c r="I51">
+        <v>3</v>
+      </c>
+      <c r="J51">
+        <v>3</v>
+      </c>
+      <c r="K51">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="1" id="{4FAB39DA-89F7-4A82-B3F6-EBBE2DAED5DE}">
+            <xm:f>A1:K45&lt;&gt;IDEAL_STRAT!A1:K45</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>A1:K51</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D00C957C-C155-4183-9431-E7332AC45C24}">
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>6</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>9</v>
+      </c>
+      <c r="J2">
+        <v>10</v>
+      </c>
+      <c r="K2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>4</v>
+      </c>
+      <c r="J13">
+        <v>4</v>
+      </c>
+      <c r="K13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14">
+        <v>3</v>
+      </c>
+      <c r="H14">
+        <v>4</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+      <c r="J14">
+        <v>4</v>
+      </c>
+      <c r="K14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>3</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>3</v>
+      </c>
+      <c r="K15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
+      <c r="K16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="F22">
+        <v>6</v>
+      </c>
+      <c r="G22">
+        <v>7</v>
+      </c>
+      <c r="H22">
+        <v>8</v>
+      </c>
+      <c r="I22">
+        <v>9</v>
+      </c>
+      <c r="J22">
+        <v>10</v>
+      </c>
+      <c r="K22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>13</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>14</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>15</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>16</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>17</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>18</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>3</v>
+      </c>
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+      <c r="I28">
+        <v>3</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>19</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29">
+        <v>3</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+      <c r="F29">
+        <v>3</v>
+      </c>
+      <c r="G29">
+        <v>3</v>
+      </c>
+      <c r="H29">
+        <v>3</v>
+      </c>
+      <c r="I29">
+        <v>3</v>
+      </c>
+      <c r="J29">
+        <v>3</v>
+      </c>
+      <c r="K29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>20</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <v>3</v>
+      </c>
+      <c r="H30">
+        <v>3</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="K30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35">
+        <v>6</v>
+      </c>
+      <c r="G35">
+        <v>7</v>
+      </c>
+      <c r="H35">
+        <v>8</v>
+      </c>
+      <c r="I35">
+        <v>9</v>
+      </c>
+      <c r="J35">
+        <v>10</v>
+      </c>
+      <c r="K35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>2</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="E36">
+        <v>2</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>3</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>5</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39">
+        <v>0</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>6</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40">
+        <v>2</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
+      <c r="G40">
+        <v>2</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>7</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41">
+        <v>2</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+      <c r="G41">
+        <v>2</v>
+      </c>
+      <c r="H41">
+        <v>2</v>
+      </c>
+      <c r="I41">
+        <v>2</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>8</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42">
+        <v>2</v>
+      </c>
+      <c r="H42">
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>2</v>
+      </c>
+      <c r="J42">
+        <v>2</v>
+      </c>
+      <c r="K42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>9</v>
+      </c>
+      <c r="B43">
+        <v>2</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43">
+        <v>2</v>
+      </c>
+      <c r="F43">
+        <v>3</v>
+      </c>
+      <c r="G43">
+        <v>3</v>
+      </c>
+      <c r="H43">
+        <v>2</v>
+      </c>
+      <c r="I43">
+        <v>2</v>
+      </c>
+      <c r="J43">
+        <v>3</v>
+      </c>
+      <c r="K43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>10</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44">
+        <v>3</v>
+      </c>
+      <c r="E44">
+        <v>3</v>
+      </c>
+      <c r="F44">
+        <v>3</v>
+      </c>
+      <c r="G44">
+        <v>3</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44">
+        <v>3</v>
+      </c>
+      <c r="K44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>11</v>
+      </c>
+      <c r="B45">
+        <v>2</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>2</v>
+      </c>
+      <c r="G45">
+        <v>2</v>
+      </c>
+      <c r="H45">
+        <v>2</v>
+      </c>
+      <c r="I45">
+        <v>2</v>
+      </c>
+      <c r="J45">
+        <v>2</v>
+      </c>
+      <c r="K45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="D50">
+        <v>4</v>
+      </c>
+      <c r="E50">
+        <v>5</v>
+      </c>
+      <c r="F50">
+        <v>6</v>
+      </c>
+      <c r="G50">
+        <v>7</v>
+      </c>
+      <c r="H50">
+        <v>8</v>
+      </c>
+      <c r="I50">
+        <v>9</v>
+      </c>
+      <c r="J50">
+        <v>10</v>
+      </c>
+      <c r="K50">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
+      </c>
+      <c r="D51">
+        <v>3</v>
+      </c>
+      <c r="E51">
+        <v>3</v>
+      </c>
+      <c r="F51">
+        <v>3</v>
+      </c>
+      <c r="G51">
+        <v>3</v>
+      </c>
+      <c r="H51">
+        <v>3</v>
+      </c>
+      <c r="I51">
+        <v>3</v>
+      </c>
+      <c r="J51">
+        <v>3</v>
+      </c>
+      <c r="K51">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="1" id="{59331A63-BA56-4A0D-8F42-207AF02F6974}">
+            <xm:f>A1:K45&lt;&gt;IDEAL_STRAT!A1:K45</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>A1:K51</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{937B308A-3064-4D2F-B194-556AEB25218E}">
   <dimension ref="A1:K51"/>

</xml_diff>

<commit_message>
cleanup of a few files & reward functions, added a new min and split model to see if the model is still learning. added an evaluation to model 14-11 in COMPARE_TO_IDEAL.xlsx
</commit_message>
<xml_diff>
--- a/startegies/COMPARE_TO_IDEAL.xlsx
+++ b/startegies/COMPARE_TO_IDEAL.xlsx
@@ -1,17 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Python\BLACKJACK-AI\BlackJack\startegies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8624736-EFBB-428D-A55C-AC4BAE7BC2D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358BEA3F-83C0-4FA3-9D35-D26FFCD67919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14385" yWindow="240" windowWidth="14250" windowHeight="15105" firstSheet="12" activeTab="14" xr2:uid="{7D4E3D51-C410-42E7-8E6F-E5B372043018}"/>
-    <workbookView xWindow="-28665" yWindow="240" windowWidth="14250" windowHeight="15105" xr2:uid="{D3AF0EBA-7B40-4C08-87C2-5ACC0D5D261F}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="15" activeTab="16" xr2:uid="{4E712069-786B-436F-9538-166F6F5D7D2C}"/>
   </bookViews>
   <sheets>
     <sheet name="IDEAL_STRAT" sheetId="1" r:id="rId1"/>
@@ -29,6 +28,8 @@
     <sheet name="strat_14_10" sheetId="13" r:id="rId13"/>
     <sheet name="strat_14_11" sheetId="14" r:id="rId14"/>
     <sheet name="strat_14_11 (2)" sheetId="15" r:id="rId15"/>
+    <sheet name="strat_15_12" sheetId="16" r:id="rId16"/>
+    <sheet name="השוואה של 14-11 מול אידיאלי" sheetId="17" r:id="rId17"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="6">
   <si>
     <t>HARD HANDS - NO PAIRS</t>
   </si>
@@ -90,12 +91,30 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -125,16 +144,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="20">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1946,22 +1982,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A2">
-    <cfRule type="expression" dxfId="17" priority="5">
+    <cfRule type="expression" dxfId="19" priority="5">
       <formula>A1:K45&lt;&gt;A1:K45</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A21:A22">
-    <cfRule type="expression" dxfId="16" priority="3">
+    <cfRule type="expression" dxfId="18" priority="3">
       <formula>A21:K65&lt;&gt;A21:K65</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A34:A35">
-    <cfRule type="expression" dxfId="15" priority="1">
+    <cfRule type="expression" dxfId="17" priority="1">
       <formula>A34:K78&lt;&gt;A34:K78</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A49:K51">
-    <cfRule type="expression" dxfId="14" priority="7">
+    <cfRule type="expression" dxfId="16" priority="7">
       <formula>A49:K93&lt;&gt;A49:K93</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9027,7 +9063,7 @@
       <c r="B6">
         <v>0</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="3">
         <v>1</v>
       </c>
       <c r="D6">
@@ -10247,6 +10283,2749 @@
       </x14:conditionalFormattings>
     </ext>
   </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E79DE841-CEF1-4ADD-9104-F501E574C3AD}">
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>6</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>9</v>
+      </c>
+      <c r="J2">
+        <v>10</v>
+      </c>
+      <c r="K2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>4</v>
+      </c>
+      <c r="K13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>3</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>3</v>
+      </c>
+      <c r="K15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
+      <c r="K16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="F22">
+        <v>6</v>
+      </c>
+      <c r="G22">
+        <v>7</v>
+      </c>
+      <c r="H22">
+        <v>8</v>
+      </c>
+      <c r="I22">
+        <v>9</v>
+      </c>
+      <c r="J22">
+        <v>10</v>
+      </c>
+      <c r="K22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>13</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>14</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>15</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>16</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>17</v>
+      </c>
+      <c r="B27">
+        <v>0</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>18</v>
+      </c>
+      <c r="B28">
+        <v>4</v>
+      </c>
+      <c r="C28">
+        <v>4</v>
+      </c>
+      <c r="D28">
+        <v>4</v>
+      </c>
+      <c r="E28">
+        <v>4</v>
+      </c>
+      <c r="F28">
+        <v>3</v>
+      </c>
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+      <c r="I28">
+        <v>4</v>
+      </c>
+      <c r="J28">
+        <v>4</v>
+      </c>
+      <c r="K28">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>19</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29">
+        <v>3</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+      <c r="F29">
+        <v>3</v>
+      </c>
+      <c r="G29">
+        <v>3</v>
+      </c>
+      <c r="H29">
+        <v>3</v>
+      </c>
+      <c r="I29">
+        <v>3</v>
+      </c>
+      <c r="J29">
+        <v>3</v>
+      </c>
+      <c r="K29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>20</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <v>3</v>
+      </c>
+      <c r="H30">
+        <v>3</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="K30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35">
+        <v>6</v>
+      </c>
+      <c r="G35">
+        <v>7</v>
+      </c>
+      <c r="H35">
+        <v>8</v>
+      </c>
+      <c r="I35">
+        <v>9</v>
+      </c>
+      <c r="J35">
+        <v>10</v>
+      </c>
+      <c r="K35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>2</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="E36">
+        <v>2</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>3</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>5</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39">
+        <v>1</v>
+      </c>
+      <c r="J39">
+        <v>1</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>6</v>
+      </c>
+      <c r="B40">
+        <v>0</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>3</v>
+      </c>
+      <c r="F40">
+        <v>3</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>7</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41">
+        <v>2</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+      <c r="G41">
+        <v>2</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>8</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42">
+        <v>2</v>
+      </c>
+      <c r="H42">
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>2</v>
+      </c>
+      <c r="J42">
+        <v>2</v>
+      </c>
+      <c r="K42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>9</v>
+      </c>
+      <c r="B43">
+        <v>2</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43">
+        <v>3</v>
+      </c>
+      <c r="E43">
+        <v>3</v>
+      </c>
+      <c r="F43">
+        <v>3</v>
+      </c>
+      <c r="G43">
+        <v>3</v>
+      </c>
+      <c r="H43">
+        <v>3</v>
+      </c>
+      <c r="I43">
+        <v>3</v>
+      </c>
+      <c r="J43">
+        <v>3</v>
+      </c>
+      <c r="K43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>10</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44">
+        <v>3</v>
+      </c>
+      <c r="E44">
+        <v>3</v>
+      </c>
+      <c r="F44">
+        <v>3</v>
+      </c>
+      <c r="G44">
+        <v>3</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44">
+        <v>3</v>
+      </c>
+      <c r="K44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>11</v>
+      </c>
+      <c r="B45">
+        <v>2</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>2</v>
+      </c>
+      <c r="G45">
+        <v>2</v>
+      </c>
+      <c r="H45">
+        <v>2</v>
+      </c>
+      <c r="I45">
+        <v>2</v>
+      </c>
+      <c r="J45">
+        <v>2</v>
+      </c>
+      <c r="K45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="D50">
+        <v>4</v>
+      </c>
+      <c r="E50">
+        <v>5</v>
+      </c>
+      <c r="F50">
+        <v>6</v>
+      </c>
+      <c r="G50">
+        <v>7</v>
+      </c>
+      <c r="H50">
+        <v>8</v>
+      </c>
+      <c r="I50">
+        <v>9</v>
+      </c>
+      <c r="J50">
+        <v>10</v>
+      </c>
+      <c r="K50">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
+      </c>
+      <c r="D51">
+        <v>3</v>
+      </c>
+      <c r="E51">
+        <v>3</v>
+      </c>
+      <c r="F51">
+        <v>3</v>
+      </c>
+      <c r="G51">
+        <v>3</v>
+      </c>
+      <c r="H51">
+        <v>3</v>
+      </c>
+      <c r="I51">
+        <v>3</v>
+      </c>
+      <c r="J51">
+        <v>3</v>
+      </c>
+      <c r="K51">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="1" id="{D01787B0-CD23-4112-8E7E-982E87DA86B6}">
+            <xm:f>A1:K45&lt;&gt;IDEAL_STRAT!A1:K45</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>A1:K51</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7563D907-53DB-47EC-84CD-32AADAB49E0C}">
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>6</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>9</v>
+      </c>
+      <c r="J2">
+        <v>10</v>
+      </c>
+      <c r="K2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>12</v>
+      </c>
+      <c r="B10" s="2">
+        <v>3</v>
+      </c>
+      <c r="C10" s="2">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2">
+        <v>4</v>
+      </c>
+      <c r="J13">
+        <v>4</v>
+      </c>
+      <c r="K13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14" s="2">
+        <v>3</v>
+      </c>
+      <c r="H14" s="2">
+        <v>4</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+      <c r="J14">
+        <v>4</v>
+      </c>
+      <c r="K14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>3</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>3</v>
+      </c>
+      <c r="K15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
+      <c r="K16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="F22">
+        <v>6</v>
+      </c>
+      <c r="G22">
+        <v>7</v>
+      </c>
+      <c r="H22">
+        <v>8</v>
+      </c>
+      <c r="I22">
+        <v>9</v>
+      </c>
+      <c r="J22">
+        <v>10</v>
+      </c>
+      <c r="K22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>13</v>
+      </c>
+      <c r="B23" s="3">
+        <v>1</v>
+      </c>
+      <c r="C23" s="3">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>14</v>
+      </c>
+      <c r="B24" s="3">
+        <v>1</v>
+      </c>
+      <c r="C24" s="3">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>15</v>
+      </c>
+      <c r="B25" s="3">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>16</v>
+      </c>
+      <c r="B26" s="3">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>17</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>18</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2">
+        <v>3</v>
+      </c>
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+      <c r="I28" s="2">
+        <v>3</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>19</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29">
+        <v>3</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+      <c r="F29" s="2">
+        <v>3</v>
+      </c>
+      <c r="G29">
+        <v>3</v>
+      </c>
+      <c r="H29">
+        <v>3</v>
+      </c>
+      <c r="I29">
+        <v>3</v>
+      </c>
+      <c r="J29">
+        <v>3</v>
+      </c>
+      <c r="K29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>20</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <v>3</v>
+      </c>
+      <c r="H30">
+        <v>3</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="K30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35">
+        <v>6</v>
+      </c>
+      <c r="G35">
+        <v>7</v>
+      </c>
+      <c r="H35">
+        <v>8</v>
+      </c>
+      <c r="I35">
+        <v>9</v>
+      </c>
+      <c r="J35">
+        <v>10</v>
+      </c>
+      <c r="K35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>2</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="E36">
+        <v>2</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36" s="2">
+        <v>0</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>3</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37" s="2">
+        <v>0</v>
+      </c>
+      <c r="H37" s="2">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38" s="4">
+        <v>1</v>
+      </c>
+      <c r="D38" s="4">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>5</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39" s="4">
+        <v>0</v>
+      </c>
+      <c r="I39" s="4">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>6</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40">
+        <v>2</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
+      <c r="G40">
+        <v>2</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>7</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41">
+        <v>2</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+      <c r="G41">
+        <v>2</v>
+      </c>
+      <c r="H41" s="2">
+        <v>2</v>
+      </c>
+      <c r="I41" s="2">
+        <v>2</v>
+      </c>
+      <c r="J41" s="4">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>8</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42">
+        <v>2</v>
+      </c>
+      <c r="H42">
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>2</v>
+      </c>
+      <c r="J42">
+        <v>2</v>
+      </c>
+      <c r="K42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>9</v>
+      </c>
+      <c r="B43">
+        <v>2</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43">
+        <v>2</v>
+      </c>
+      <c r="F43" s="2">
+        <v>3</v>
+      </c>
+      <c r="G43">
+        <v>3</v>
+      </c>
+      <c r="H43">
+        <v>2</v>
+      </c>
+      <c r="I43">
+        <v>2</v>
+      </c>
+      <c r="J43">
+        <v>3</v>
+      </c>
+      <c r="K43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>10</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44">
+        <v>3</v>
+      </c>
+      <c r="E44">
+        <v>3</v>
+      </c>
+      <c r="F44">
+        <v>3</v>
+      </c>
+      <c r="G44">
+        <v>3</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44">
+        <v>3</v>
+      </c>
+      <c r="K44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>11</v>
+      </c>
+      <c r="B45">
+        <v>2</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>2</v>
+      </c>
+      <c r="G45">
+        <v>2</v>
+      </c>
+      <c r="H45">
+        <v>2</v>
+      </c>
+      <c r="I45">
+        <v>2</v>
+      </c>
+      <c r="J45">
+        <v>2</v>
+      </c>
+      <c r="K45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="D50">
+        <v>4</v>
+      </c>
+      <c r="E50">
+        <v>5</v>
+      </c>
+      <c r="F50">
+        <v>6</v>
+      </c>
+      <c r="G50">
+        <v>7</v>
+      </c>
+      <c r="H50">
+        <v>8</v>
+      </c>
+      <c r="I50">
+        <v>9</v>
+      </c>
+      <c r="J50">
+        <v>10</v>
+      </c>
+      <c r="K50">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
+      </c>
+      <c r="D51">
+        <v>3</v>
+      </c>
+      <c r="E51">
+        <v>3</v>
+      </c>
+      <c r="F51">
+        <v>3</v>
+      </c>
+      <c r="G51">
+        <v>3</v>
+      </c>
+      <c r="H51">
+        <v>3</v>
+      </c>
+      <c r="I51">
+        <v>3</v>
+      </c>
+      <c r="J51">
+        <v>3</v>
+      </c>
+      <c r="K51">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
cleaned up trainers, trained new min model 16 and split 13.
</commit_message>
<xml_diff>
--- a/startegies/COMPARE_TO_IDEAL.xlsx
+++ b/startegies/COMPARE_TO_IDEAL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Python\BLACKJACK-AI\BlackJack\startegies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358BEA3F-83C0-4FA3-9D35-D26FFCD67919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A881E47-931F-4760-A4EA-9F458FF4DA75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="15" activeTab="16" xr2:uid="{4E712069-786B-436F-9538-166F6F5D7D2C}"/>
+    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11295" firstSheet="15" activeTab="17" xr2:uid="{4E712069-786B-436F-9538-166F6F5D7D2C}"/>
   </bookViews>
   <sheets>
     <sheet name="IDEAL_STRAT" sheetId="1" r:id="rId1"/>
@@ -30,6 +30,7 @@
     <sheet name="strat_14_11 (2)" sheetId="15" r:id="rId15"/>
     <sheet name="strat_15_12" sheetId="16" r:id="rId16"/>
     <sheet name="השוואה של 14-11 מול אידיאלי" sheetId="17" r:id="rId17"/>
+    <sheet name="strat_16_13" sheetId="18" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="6">
   <si>
     <t>HARD HANDS - NO PAIRS</t>
   </si>
@@ -13029,6 +13030,1386 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{359E5BA0-583C-45C8-BA09-246EFA7B18AD}">
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>6</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>9</v>
+      </c>
+      <c r="J2">
+        <v>10</v>
+      </c>
+      <c r="K2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>4</v>
+      </c>
+      <c r="K13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>3</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="J15">
+        <v>3</v>
+      </c>
+      <c r="K15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
+      <c r="K16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="F22">
+        <v>6</v>
+      </c>
+      <c r="G22">
+        <v>7</v>
+      </c>
+      <c r="H22">
+        <v>8</v>
+      </c>
+      <c r="I22">
+        <v>9</v>
+      </c>
+      <c r="J22">
+        <v>10</v>
+      </c>
+      <c r="K22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>13</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>14</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>15</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>16</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>17</v>
+      </c>
+      <c r="B27">
+        <v>4</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>4</v>
+      </c>
+      <c r="I27">
+        <v>4</v>
+      </c>
+      <c r="J27">
+        <v>4</v>
+      </c>
+      <c r="K27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>18</v>
+      </c>
+      <c r="B28">
+        <v>4</v>
+      </c>
+      <c r="C28">
+        <v>4</v>
+      </c>
+      <c r="D28">
+        <v>4</v>
+      </c>
+      <c r="E28">
+        <v>4</v>
+      </c>
+      <c r="F28">
+        <v>4</v>
+      </c>
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+      <c r="I28">
+        <v>4</v>
+      </c>
+      <c r="J28">
+        <v>4</v>
+      </c>
+      <c r="K28">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>19</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29">
+        <v>3</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+      <c r="F29">
+        <v>3</v>
+      </c>
+      <c r="G29">
+        <v>3</v>
+      </c>
+      <c r="H29">
+        <v>3</v>
+      </c>
+      <c r="I29">
+        <v>3</v>
+      </c>
+      <c r="J29">
+        <v>3</v>
+      </c>
+      <c r="K29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>20</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <v>3</v>
+      </c>
+      <c r="H30">
+        <v>3</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="K30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35">
+        <v>6</v>
+      </c>
+      <c r="G35">
+        <v>7</v>
+      </c>
+      <c r="H35">
+        <v>8</v>
+      </c>
+      <c r="I35">
+        <v>9</v>
+      </c>
+      <c r="J35">
+        <v>10</v>
+      </c>
+      <c r="K35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>2</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>3</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>5</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39">
+        <v>1</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>6</v>
+      </c>
+      <c r="B40">
+        <v>0</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>3</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>7</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41">
+        <v>2</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+      <c r="G41">
+        <v>0</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>8</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42">
+        <v>2</v>
+      </c>
+      <c r="H42">
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>2</v>
+      </c>
+      <c r="J42">
+        <v>2</v>
+      </c>
+      <c r="K42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>9</v>
+      </c>
+      <c r="B43">
+        <v>2</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43">
+        <v>2</v>
+      </c>
+      <c r="F43">
+        <v>3</v>
+      </c>
+      <c r="G43">
+        <v>3</v>
+      </c>
+      <c r="H43">
+        <v>3</v>
+      </c>
+      <c r="I43">
+        <v>3</v>
+      </c>
+      <c r="J43">
+        <v>3</v>
+      </c>
+      <c r="K43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>10</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="D44">
+        <v>3</v>
+      </c>
+      <c r="E44">
+        <v>3</v>
+      </c>
+      <c r="F44">
+        <v>3</v>
+      </c>
+      <c r="G44">
+        <v>3</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44">
+        <v>3</v>
+      </c>
+      <c r="K44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>11</v>
+      </c>
+      <c r="B45">
+        <v>2</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>2</v>
+      </c>
+      <c r="G45">
+        <v>2</v>
+      </c>
+      <c r="H45">
+        <v>2</v>
+      </c>
+      <c r="I45">
+        <v>2</v>
+      </c>
+      <c r="J45">
+        <v>2</v>
+      </c>
+      <c r="K45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="D50">
+        <v>4</v>
+      </c>
+      <c r="E50">
+        <v>5</v>
+      </c>
+      <c r="F50">
+        <v>6</v>
+      </c>
+      <c r="G50">
+        <v>7</v>
+      </c>
+      <c r="H50">
+        <v>8</v>
+      </c>
+      <c r="I50">
+        <v>9</v>
+      </c>
+      <c r="J50">
+        <v>10</v>
+      </c>
+      <c r="K50">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
+      </c>
+      <c r="D51">
+        <v>3</v>
+      </c>
+      <c r="E51">
+        <v>3</v>
+      </c>
+      <c r="F51">
+        <v>3</v>
+      </c>
+      <c r="G51">
+        <v>3</v>
+      </c>
+      <c r="H51">
+        <v>3</v>
+      </c>
+      <c r="I51">
+        <v>3</v>
+      </c>
+      <c r="J51">
+        <v>3</v>
+      </c>
+      <c r="K51">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="1" id="{039DBDAB-8CA4-483F-877A-3A5002220162}">
+            <xm:f>A1:K45&lt;&gt;IDEAL_STRAT!A1:K45</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>A1:K51</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{937B308A-3064-4D2F-B194-556AEB25218E}">
   <dimension ref="A1:K51"/>

</xml_diff>